<commit_message>
strict cleanup pass per reviewer feedback: drop low-substance reactions and near-duplicates
</commit_message>
<xml_diff>
--- a/Topic Relevant Comments/Nigeria/Agba John Doe_Never Leave Marriage Because Husband Cheated.xlsx
+++ b/Topic Relevant Comments/Nigeria/Agba John Doe_Never Leave Marriage Because Husband Cheated.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="201">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="116" uniqueCount="116">
   <si>
     <t>text</t>
   </si>
@@ -22,9 +22,6 @@
     <t>This is why, when I go on dates. I ask a lot of questions. What's your take on infidelity? Is it possible to stay faithful in a marriage? I'm not saying one cannot fall, but I won't go for someone who already has it in mind to cheat or believes it's normal, even before marrying.</t>
   </si>
   <si>
-    <t>A man is who provides &amp; protects . A loyal man is a disciplined man</t>
-  </si>
-  <si>
     <t>"Except you're done with marriage for good &amp; don't wish to be married again." I belong to this school of thought. For me, infidelity is one of the unpardonable sins.</t>
   </si>
   <si>
@@ -34,21 +31,9 @@
     <t>But can we tell men to shun cheating/infidelity?? If you still want to mess around then why marry?</t>
   </si>
   <si>
-    <t>Key point: A man can be faithful because he's disciplined and not be a good husband and wife. A man can be a cheat but be a responsible father to his wife and children. More wisdom sir</t>
-  </si>
-  <si>
     <t>The African society is very "patriarchal"; when it comes to marriage, men who have the wherewithal to provide stability and security are the prize. If a woman leaves the "prize" on account of infidelity in marriage, he'll have a lot of fine options to choose from if he wishes...</t>
   </si>
   <si>
-    <t>'Glorifying cheating??' In the past men were bold enough to marry more than 1 &amp; it wasn't really about 'sex'. And this was across cultures all around the world. Then came the wave of radical feminism who demanded one man-one wife. 1/</t>
-  </si>
-  <si>
-    <t>Islaam solves this problem. A cheating husband or wife is not a choice at all if they are unrepentant. The man can always get someone to marry, the woman too can always get. A man has a chance of marrying four. She may marry another virtuous man as a as a 2nd or 3rd wife.</t>
-  </si>
-  <si>
-    <t>For women, the demographics aren't in their favor. For every male baby delivered, many hundreds of females are available not to mention the age difference among spouses and yet the males aren't all available for marriage due to mental illness and incarceration.</t>
-  </si>
-  <si>
     <t>Sadly, this is the truth. But men should not see this as a license to cheat. There is no need to betray the love of your partner. Be committed and do whatever you can to make relationship/marriage work.</t>
   </si>
   <si>
@@ -58,15 +43,6 @@
     <t>What would be reduce from the life span of a man, if he decides to be a faithful husband? Can't they see their wife's are hurting and yet they derive pleasure in increasing the hurt with the excuse of "men are polygamous in nature" ‍♀️</t>
   </si>
   <si>
-    <t>Both men and Women have that potential of cheating or not totally being faithful to their Spouse..Just that it's been done in their different stages of their life, which is their prime stages. At a woman's prime stage, that's when she is still young and probably haven't married..</t>
-  </si>
-  <si>
-    <t>Morale of the story No body should cheat! No body also should stay with a partner that cheats for their sanity sake. Gender balance roles 50/50 by God grace and for conscience sake I have no intentions to cheat on my husband My husband will not cheat on me. So help us God!</t>
-  </si>
-  <si>
-    <t>Married men please stop cheating on your spouse</t>
-  </si>
-  <si>
     <t>It's the way they glorify cheating and marriage sis. What about the woman's mental health?</t>
   </si>
   <si>
@@ -82,21 +58,9 @@
     <t>Because of this narrative, a lot of marriages in those days were loveless, the women stayed because they wanted to remain married And most of them did not have where to go or any means to survive outside marriage. But this narrative is changing.</t>
   </si>
   <si>
-    <t>And the fool that cheated would get a loyal virgin or woman abi? Oga pack well there is no valid truth in what you have said so far. Before getting married ask yourself why. Go to the school of marriage learn because it's an institution with lots of hurts</t>
-  </si>
-  <si>
     <t>Which means it is a man's world after all. Men get away with cheating, women don't. Why? Because men are allowed to be irresponsible but women are held to high standards. On that note, it would be a fact to say men are raised to kill and women raised to survive.</t>
   </si>
   <si>
-    <t>This isn't about wokeness can ll atleast stop glorying cheating ‍♀️ I don't see why u men can't stay faithful ‍♀️Do you even know how ll ladies feel knowing our man is cheating on us ‍♀️ men should do better unna no be God</t>
-  </si>
-  <si>
-    <t>Chai! This marriage thing isn't for the faint hearted</t>
-  </si>
-  <si>
-    <t>Yes sir since being faithful is a farce let us stay with cheating men in peace,till they give us HIV or marry the side chick and be spiting us on social media with it,you too get sense walai</t>
-  </si>
-  <si>
     <t>Please..a woman who intend to get married and stay committed to it should read this tweet with all sense of sincerity &amp; open mind. Especially where sir Jon said THE CONSEQUENCES ARE NOT THE SAME FOR BOTH GENDER.</t>
   </si>
   <si>
@@ -109,33 +73,21 @@
     <t>"A man does not cheat on you because he doesn't find you valuable anymore" Dear Sister, if U believe in marriage please fight for it, consequences of cheating are not the same for a man and woman As the woman you know the odds are against you, don't let SM deceive you</t>
   </si>
   <si>
-    <t>This is a hard truth for feminist to comprehend.</t>
-  </si>
-  <si>
     <t>This is one falsehood propergated by men to lock women who are unhappy in their marriages due to a cheating spouse. Forgiveness should be done for one's healing but staying is a choice you cannot stay with a serial cheater because he is purportedly the best.</t>
   </si>
   <si>
     <t>TRUTH! but please balance it a lil, so that some men who lack understanding of what it takes to make marriage work dont go about sleeping on anything on skirt and rubbing it to their wives face. Men have better options after divorce but need to show effort to make the union work</t>
   </si>
   <si>
-    <t>Hmmmm dis thread no sit well wit d woke queens but in all i believe men can still be faithful to their wives...but wetin i sabi sef? It is what it is</t>
-  </si>
-  <si>
     <t>Might it be difficult for a woman to find another husband after marriage? Yes it might. Dat doesn't mean she should stay and condone cheating till he infects her with diseases or she dies from heartbreak &amp; depression. Statements like dis tend 2 make it seem right for men to cheat</t>
   </si>
   <si>
-    <t>The summary is husband no dey outside. Abi. Man can cheat and still love and respect the house wife. No be say cheating good o. Women has the power to stop a man from cheating, but them no dey calm down.</t>
-  </si>
-  <si>
     <t>African men seem to read a different Bible when it comes to adultery, it's the woman I will hold , if you stay and get some incurable std , and you both die and leave innocent children that you brought into this world ,you memories will be cursed. Choose wisely.</t>
   </si>
   <si>
     <t>I have seen a lot of married women leave there husband cause of cheating and later they start dragging people's husband or being side chick and I keep wondering why they left their marriage in the first place . Sir my question is what if the man keeps giving the wife infection?</t>
   </si>
   <si>
-    <t>The cheating or infidelity or I'll rather say polygamy is in the DNA of men originally designed and created by God are you ready to recreate another man ? Are you GOD?</t>
-  </si>
-  <si>
     <t>I see a lot of men happily replying and seconding this tweet, now the tweet itself is a sad reality meaning that it holds true for majority. If you truly love your woman , you stay faithful, it breaks a woman and a lot of you can't even take it if your woman cheats on you,</t>
   </si>
   <si>
@@ -160,9 +112,6 @@
     <t>Many women who left their marriage becos of cheating are now cheating with another women's husbands. What a shame. It better to be the first than to be the second or third options due to impatient and lack of wisdom. "Never leave a hot trying pan to fire" it not funny outside.</t>
   </si>
   <si>
-    <t>Ye lots that projects marriage as if men are doing women favor by being married to them. Motivational speaker wanna be.</t>
-  </si>
-  <si>
     <t>Let me give u an original answer.Originally god never created man 2 b one man &amp;one woman.monogamy is a Western construct.A woman cant stand the libido of an average man. So from the biblical evidence will have more telling of that men in the Bible married so many women</t>
   </si>
   <si>
@@ -175,15 +124,6 @@
     <t>At first when I began to read, it makes sense. Mr. John with all due respect, it will be respectful to women to encourage them to stay committed to their marriage for more Godly reasons, e.g; none of our Godly mother like Sarah left Abraham for cheating. Infact, I say this a lot,</t>
   </si>
   <si>
-    <t>If he cheats on you. Just leave him with the kids and be the one paying child maintenance. That way you'll have the ability to move as you please. He can raise the kids with his new wife. While they visit you over the weekends. ❤️</t>
-  </si>
-  <si>
-    <t>At the end those side chics would still leave you,and that's for a fact.I've always said this and I'll keep saying it " an average male child is not properly trained" why would you be married and all you can think of is how to betray your familyGod pls help me be a good husband</t>
-  </si>
-  <si>
-    <t>Thanks bro, u nailed it✅ I pray God should give me more patient in marriage when i marry</t>
-  </si>
-  <si>
     <t>Be calm pretty posh, Nobody is glorifying CHEATING HERE... Have you ever asked yourself why MEN can marry as many women as them like but a WOMAN can't marry many MEN as she can If you can answer the question, then FINE</t>
   </si>
   <si>
@@ -193,48 +133,24 @@
     <t>Well said John, sad reality....as much as you have a lot to say about these female gender also teach the men DISCIPLINE for once see if you can step out of the prejudice against women and speak from a place of good humanity a lot of unfairness is done to the female gender.</t>
   </si>
   <si>
-    <t>90% of men can't stay faithful to one pussy, it's really bad, very bad, but that's just reality</t>
-  </si>
-  <si>
     <t>Can the man also forgive his wife?</t>
   </si>
   <si>
-    <t>As silly and as primitive as it may sound, its still a man's world. Nature itself is unfair to women, but it is what it is</t>
-  </si>
-  <si>
     <t>There are Million ways to deal with a cheating husband without cheating back or divorcing him. U can't continually do someone dirty &amp; expect to live a beautiful life ur wife can be ur KARMA &amp; more when she chooses to She having a source of income &amp; kids, is just d icing on d cake</t>
   </si>
   <si>
     <t>Societal patriarchy! Does it make it right?</t>
   </si>
   <si>
-    <t>Everybody getting the man and woman thing wrong. Marriage and relationships will continue to be a fail or even worse if we continue like This</t>
-  </si>
-  <si>
     <t>A girl I know was in a serious relationship with a guy. They were close to marriage. Then she found out he cheated on her with another girl. She left him. He got married to his side chic. Now his former fiancee is now his side chic. While the former side chic is now the wife.</t>
   </si>
   <si>
-    <t>Well just know , if you agree with this thread you must agree to accept bastard children , or agree with the possibility of getting HIV there's no point enduring cheating for 20 years just to leave when they bring the results of the cheating , accept all with full chest good wife</t>
-  </si>
-  <si>
-    <t>If you trust your physical appearance and under 30, divorce. if you can't stand a cheating husband, divorce. Especially if he is rich, take all u can. Even more, if he is poor. You will find another man for sure. What I can't guarantee is whether that new man will cheat or not.</t>
-  </si>
-  <si>
     <t>Most people here saying woman should fight for their marriages,as if she is the only one involved in the institution. Y can't men fight to keep the marriage. Or are they fighting there own through cheating? SMH.</t>
   </si>
   <si>
-    <t>I expect many ladies won't like this, but unfortunately, this is the reality of the society we live in. It really is a man's world out here.</t>
-  </si>
-  <si>
-    <t>Leave judgment day to God and do what you have to do now for marriage's sake, that's if you want to.</t>
-  </si>
-  <si>
     <t>Dear women,don't listen to this ...if you're married to a cheating man and your mental health can't take it..please leave...there's nothing more important than peace of mind...Marraige is not a do or die affair ,don't stay in an unhappy marriage because you want to be called Mrs</t>
   </si>
   <si>
-    <t>A man can cheat and still love his wife but if a woman cheat she lost respect for the husband</t>
-  </si>
-  <si>
     <t>Women are not 2nd class citizens with no choice. Many women have caught diseases, bn killed, kids destroyed cause of cheating. Protect yourself &amp; ur kids Queen. You are worth being faithful to. Nobody is doing you a favor. There are stil good men out there. Just do you &amp; be hapy</t>
   </si>
   <si>
@@ -244,57 +160,27 @@
     <t>I remember a story I read here, of a wife who divorced because she found out he cheated. Man married side girl in no time. Former wife came to beg, dude said he moved on but she can be his side piece- she agreed</t>
   </si>
   <si>
-    <t>Is this applicable to those that are dating?</t>
-  </si>
-  <si>
-    <t>My dear, Men are the God you see on Earth. Even the different religions books affirms that your husband is your Lord &amp; Master. E get why e be like that. It's been that way before dem born you and me. End.</t>
-  </si>
-  <si>
     <t>There has to be some sort of punishment for cheating so men don't do it bcos they knw they operate frm a more favourable spectrum, to avoid a mentality of "what can she do" "she can't leave" " she knows no man will marry her again" "power lies with me". Women are at the receiving</t>
   </si>
   <si>
-    <t>I shake my head at men that will take this as an initiative to cheat or continue cheating on their wives</t>
-  </si>
-  <si>
     <t>Hate it all u want, this is the stark reality of Nigeria. It is VERY WRONG and shouldn't be so. Nonetheless, women try get your money to avoid a lot of the aforementioned fuckery because it seems finance has a lot to do with this. As a male, BE A FAITHFUL AND GOOD HUSBAND!!!!</t>
   </si>
   <si>
-    <t>I don't support cheating by any means but a psychologist on TEDX once said that; Men cheat to KEEP their marriage, WOMEN cheat to leave their marriage. A man just need a place to cheat, but women need a reason to cheat. That's why a cheating woman should never be let back in.</t>
-  </si>
-  <si>
     <t>Sadly true, but I can't help think that this only just adds to giving some men the license and validity to cheat, rub it in the face of the wife and expect her to persevere because she can be easily replaced.</t>
   </si>
   <si>
     <t>And sincerely this is one of the beauty of salvation.. No believing man will cheat on you.. It's not about morals for such a man rather it's about eternal life and self worth. Joseph(s) don't fall for beauties no matter the shapes. They consider it a sin against God..</t>
   </si>
   <si>
-    <t>That's bitter truth , but men can do better and work on their self discipline. Because the women have started to cheat back which leads to " men bringing up children that are not theirs " DNA palaver up and down</t>
-  </si>
-  <si>
-    <t>I just feel in as much as your marriage is peaceful, accomodating, everything is going on smoothly and u r happy as a lady in it, don't seek for a second. I know how painful and frustrating it can be if you see your partner cheating, but if he doesn't do it in from of u, or he</t>
-  </si>
-  <si>
     <t>this comment! like they think all women can endure cheating..my dad was a serial cheat and i know how my mum was feeling before she died..and i can never ever endure like my mum..never!i will rather be alone than endure nonsense..my happiness and my sanity comes first.</t>
   </si>
   <si>
-    <t>So in other words, cheating is healthy and men should do it more?? Or they should still try and be decent with their ways??</t>
-  </si>
-  <si>
-    <t>So what about situation were the cheating partner get his /her partner infected of a STD???</t>
-  </si>
-  <si>
     <t>Every next generation makes the mistake of assuming they are smarter than the previous ones. There are curtains that would have protected women socially that women have ripped off now. It's gender equality, may the best human win.</t>
   </si>
   <si>
     <t>Majorly men cheat because they don't get what they want from their women and they can't change them to what they want. In some cases you will find out that the man married the body he desire but not the soul he wanted. Then he would go in search of the one that suit his fantasy</t>
   </si>
   <si>
-    <t>Women and men will never be the same.. This will forever exist without going into extinction. Just like saying racism will stop, we all know surely it will exist directly or indirectly. Men will always cheat no matter what! 98% of rich married men cheats..</t>
-  </si>
-  <si>
-    <t>Are you encouraging men to keep cheating ?</t>
-  </si>
-  <si>
     <t>Just by reading comments, men feel happy that u ve made this thread. Women who wish to remain committed to their cheating partner must learn to substitute love for money/wealth. If ur hubby doesn't cater for u/children and u do not earn more by being married, please leave!</t>
   </si>
   <si>
@@ -304,9 +190,6 @@
     <t>Clearly it is evident in our societal response. Omo it require deep thoughts before a woman must leave her marriage otherwise she'll end up regretting her actions for the rest of her entire life if she can't find what she once had, and the reality that she can never find it. Hmm</t>
   </si>
   <si>
-    <t>Who do men cheat with? Is it not women.</t>
-  </si>
-  <si>
     <t>While I find everything written here understandable, I still think a cheating husband deserves some kind of punishment from his wife. At least something to make him not want to do it another time. Repeating this act is however evil and shouldn't be seen as normal no matter what.</t>
   </si>
   <si>
@@ -322,9 +205,6 @@
     <t>You definitely deserve happiness and someone who is faithful and loyal to you,not a man that would say,men are allowed to cheat not a woman..your life would definitely be better and you'll still end up finding someone who appreciates your worth.</t>
   </si>
   <si>
-    <t>When we men were growing up no woman wanted us , we remaind faithful to our dreams when you women were young every man wanted you that was why you women find it difficult to commit to a man during your prime cause you had so many options some even cheated but we maintained cool</t>
-  </si>
-  <si>
     <t>This kind of mentality is the reason why men often get away with there shameless deeds while women are prone to emotional and shameful attacks. Men that cannot control there erection, are expecting women to abide with them forever, what a joke. Women run ooh, don't die in silence</t>
   </si>
   <si>
@@ -334,24 +214,12 @@
     <t>This tweet shows it's really a shame on men. So irresponsible that they cannever bring up a set of responsible men. I wish men's eyes will be opened to damages they indirectly cause their children by their irresponsible acts. What a shame. Kudos. You can cheat on.</t>
   </si>
   <si>
-    <t>Now we men have approached our prime and mostly every woman wants us and you ladies have expired no man wants you and you now wants us to remain faithful because the table has turned. Lolzzzzzzz</t>
-  </si>
-  <si>
-    <t>Hope the man won't leave when he discovers that the woman cheated</t>
-  </si>
-  <si>
     <t>Ahh mentor no oo i no agree with this one Instead let's beckon on the men to do better and remain ever faithful</t>
   </si>
   <si>
     <t>Wow!!! What a world we live in. So on judgement day, The men will judge differently because said it's ok for men to cheat because it's a reality. so if you encourage men to be faithful, the world will end and it's a sad reality. Please we can do better.</t>
   </si>
   <si>
-    <t>Men are naturally polygyny. The earlier you understand this, the better it is for you. I'm looking for a second wife oooo. I don't cheat and I can't cheat. My pencil will not enter any hole except my wives</t>
-  </si>
-  <si>
-    <t>Please what's your perspective about cheating.. like I'd really love to know.. i ask bcos you're a lady.</t>
-  </si>
-  <si>
     <t>Call me weird but I've never really seen cheating as a basis for calling off a relationship. There's more to a relationship than sex. Just saying, people hold sex more dare than the relationship itself.</t>
   </si>
   <si>
@@ -367,54 +235,27 @@
     <t>Woke Queens will feel that SIR JD is a woman hater but in truth he's said it all. A man @ 70 can marry a virgin but a woman can't. The patient/strong willed wife can change her cheating husband 4d better. You think other men are better than your husband, wait for a shocker.</t>
   </si>
   <si>
-    <t>That's the way it is..the consequences of cheating are never the same, take it or leave it</t>
-  </si>
-  <si>
-    <t>A man cheats due to what going on around him but women cheat due to their lack reasoning after you were told you were created from a rib in the man's body do you know if the man's rib created more than 4women</t>
-  </si>
-  <si>
     <t>You preach and encourage men to cheat because it's reality. Why not open an organization where we encourage thieves and murderers because it's a reality? Regardless of gender, let's treat others how we would want to be treated and love. There's no crown for cheating!!!</t>
   </si>
   <si>
     <t>Most times when people call off relationships, it's not just the cheating, there's more</t>
   </si>
   <si>
-    <t>Testosterone na your mate? Imagine your wife is on birth control pills which reduces the release of their sex hormones but your Testosterone is running on auto pilot. Every morning you wake up with hard dick. You're a ticking time bomb to the fidelity world. That's where</t>
-  </si>
-  <si>
     <t>Lesson: don't leave your man/husband because of rain, it rains everywhere. This is just reality of life. I can't fight or leave because of another woman, I believe he is an adult and he knows what is good for him.</t>
   </si>
   <si>
-    <t>I know of a wife who was too feminist. The guy went on to put a ring on his side chick and the first wife with a traditional marriage is now the side chick. He visits her here n there</t>
-  </si>
-  <si>
-    <t>It's what it is..Irony of life and it's D fact. Imagine leaving Ur cheating husband. Ladies it rain everywhere oh. Don't let any feminist motivational speaker talk you to abandoning Ur home.Becos the reality of it all is that you will always Be D side Chic or remain single 4 life</t>
-  </si>
-  <si>
     <t>What exactly is everything a woman will lose? She has her life, dignity, self-esteem and can mostly take care of herself. Should she then ignore her emotions and live without peace of mind or as it is "heartache" for the sake of marriage?</t>
   </si>
   <si>
     <t>That's why divorce laws should be reviewed in Nigeria....By the time you think of losing half your shxt, you'll reconsider cheating</t>
   </si>
   <si>
-    <t>I like to put it simple: A man will not cheat on you, not because he loves you but out of RESPECT for (1) himself &amp; (2) you. Hence, a man who loves you will take a bullet for you from a lady he is cheating on you with.</t>
-  </si>
-  <si>
-    <t>John have jxt explained everything to d dust oga na oga joh dat is jxt it,a man can cheat and still love and respect his wife but can't say so for a woman dats y d repercussion ain't d same sha</t>
-  </si>
-  <si>
     <t>The cost-benefit analysis comes to play. If she cheats on her man for short-term reasons, she cheats herself on the long-run. If she leaves her man, there are legion of thirsty women waiting to descend on her man. The man will lose his wife. The woman will lose everything.</t>
   </si>
   <si>
-    <t>I see comments here from men who absolutely know nothing of what they are talking about, but go on cos they want to score cheap points with ladies in the Cs. Men and Women privileges differ, men don't crave women privileges, but women want men privileges. Witchcraft, simple!</t>
-  </si>
-  <si>
     <t>Na una sabi. It is dangerous to stay with a cheating man, even if not for your ego at least for your health. Make him no go carry disease come home poor woman wey dey mind her business for house. To your tents o Israel!</t>
   </si>
   <si>
-    <t>What's all this one now? Marriage na by force?</t>
-  </si>
-  <si>
     <t>He didn't glorify cheating nah! He's said several times that it's not good. The point of the tweet is to advice not to be quick to leave because of societal and individual standards. A lot of things as sad as they sound are actually true!</t>
   </si>
   <si>
@@ -424,30 +265,15 @@
     <t>I had woke thoughts until I realised that I just didn't want to accept the painful things said. That some realities are painful makes them no less realities. I would choose to be celibate if I find myself with a cheating husband. They're not worth being sad in a union.</t>
   </si>
   <si>
-    <t>Not only married women. Dating women too. The more "exes" you're accumulating. The lesser the men that finds interest in you.</t>
-  </si>
-  <si>
-    <t>Yes sir, u just reveal the whole truth about inter sexual relationship. Women can never be like men. Men are polygamous in nature, and don't forget men are always horny due to high testosterone.</t>
-  </si>
-  <si>
     <t>It's very funny how people think. So what if this said husband is late sef, won't the woman survive??? Why do men feel women should be cheated on as a right? How will you father's feel if your little girl gets married and the husband turns out to push her to depression???</t>
   </si>
   <si>
     <t>Last 2 years my neighbor's wife left because she noticed that he cheated. Not long after that lockdown start baba start making out with another lady in the next compound words got to the wife where she was staying with her family at ikorodu babe return baba say he no marry again</t>
   </si>
   <si>
-    <t>I always ask, if all men cheat or all men are dogs why will u leave your man for another man?</t>
-  </si>
-  <si>
     <t>The problem is with we"African men"who's got to do better not you,And that mentality of all men cheat needs to be changed because this stupid mentality is passed down to the younger ones,I feel it's time we start to teach and encourage ourselves as men to be better for our family</t>
   </si>
   <si>
-    <t>Don't let anyone; whether on the internet or family and friends, tell you what to do. I've seen faithful married women now suffering from AIDS given to them by their promiscuous community penis husbands. Don't let anyone tell you anything. Weigh your life and take your decision.</t>
-  </si>
-  <si>
-    <t>John Doe will always say "men don't cheat with ghost" emotionally triggered people will not see where he wrote that "if you're done with the marriage,you can leave a cheating man".</t>
-  </si>
-  <si>
     <t>And do u men seat and think about the pain and trauma you're putting ur innocent wife through? How do u comfortably hurt a woman u claim to love? Omo I'm not built emotionally for this o and hubby knows, if he ever cheats,it will completely destroy me</t>
   </si>
   <si>
@@ -457,27 +283,15 @@
     <t>Lol. I'm just happy that women are slowly beginning to be independent and choosy. Because this was legit the scum they fed our mothers. Thats why sugar daddy is now a culture. Grown, married, men disgustingly preying on young girls while leaving their wives miserable</t>
   </si>
   <si>
-    <t>When he had a thread about women being committed to their emotions and not men's sacrifices, the women were clapping for him. Now that he has also talked about reality of the consequences of cheating not being the same for a man and a woman una wan chop am raw!! .. Choo!! ‍♂️</t>
-  </si>
-  <si>
     <t>I ask again....if she decides to leave will she remain celibate? If not who will she pick? A younger man who will be faithful to her? Another man who will carry all her responsibilities and be faithful to her?.... If your answer is same as he has typed, then he's not wrong.</t>
   </si>
   <si>
     <t>I honestly hate to admit that this thread is true. I just hope that something can happen to our cultures to bring women out of this shackles. I know a lovely woman who is suffering as a result of this. In her own case the man left her. Honestly, I rub the shame on d faces of men.</t>
   </si>
   <si>
-    <t>Most divorced women of African descent end up bring past around like footballs while the man ends up in a stable relationship/marriage. Don't leave your husband for the streets sistas‍♂️‍♂️‍♂️</t>
-  </si>
-  <si>
     <t>Truth, we had this argument on a women group once, myself and some women are of this opinion, not everything divorce your husband and after divorce you will become the reason you left your home in another woman's marriage. A divorce woman can rarely marry a fresh man but some...</t>
   </si>
   <si>
-    <t>We've heard you sir There's no problem just keep this same energy when your sister gets cheated on and probably gets and STI from her husband</t>
-  </si>
-  <si>
-    <t>Value sir .....thank u for this community I have be able to learn a lot Men and women does not have the same grace when dey cheat</t>
-  </si>
-  <si>
     <t>This is the sad reality. There was this man in our business line he was cheating on the wife then one of his boys told the wife and the wife confronted the husband shouting, threatening and all that, the moment the man found out who told her he first of all sent the boy away</t>
   </si>
   <si>
@@ -487,102 +301,45 @@
     <t>I wonder why I will leave my husband on the account of cheating on me only to go and settle down as a Second wife to another man or a side chick, woman make una dey apply sense for matter like cheat make number 1no turn to number 2 sake of say you dey vex</t>
   </si>
   <si>
-    <t>Ladies that has slept with multiple dicks before marriage is also complaining about enduring the marriage. If as a lady you'd married as a virgin then your complaining is valid. Others should be grateful to God and the man for considering them worthy to be called a wife.</t>
-  </si>
-  <si>
     <t>How is a woman supposed to stop a man from cheating? Is she supposed to flog him? How? So as an adult man that you are, you realize that cheating is not good but you continue and then you're expecting the woman to be to the one stop you. Why can't you stop yourself? Na wah o.</t>
   </si>
   <si>
     <t>Husband get protected, If you choose to stay please get tested frequently too. Recently came across a petition where the husband infected the wife wit HIV, her family had to speak to her to stay since they were both infected and sent the kids off abroad so dy don't get infected.</t>
   </si>
   <si>
-    <t>A thread like this resonates with life and reality, you can't find this undiluted truth anywhere, if you like heed to it, if you like don't, it's either you learn to live or live to perish.</t>
-  </si>
-  <si>
-    <t>He's not encouraging men to cheat. It's a sad reality</t>
-  </si>
-  <si>
-    <t>God please hide me from men that glorify cheating</t>
-  </si>
-  <si>
-    <t>Please how about a man that cheats and beat his wife what should the woman do</t>
-  </si>
-  <si>
     <t>This is not 1809 . This 2022 and women have options now. Women with dead husbands take care of their children alone but you want a woman to stay with a cheating one for kids,when most of these women are even the breadwinner in the family</t>
   </si>
   <si>
-    <t>Find out if he's cheating with 9in10.com, then leave Sis</t>
-  </si>
-  <si>
     <t>I read the write up till the end, not all your points are valid man, you're making it sound like African women are very primitive... But your view towards women make me feel like you think they lack self esteem... Everyone has his or her marital story don't make it sound like a</t>
   </si>
   <si>
-    <t>... Are you now saying, even in a abusive marriage, make she stay, abusive marriage dat de husband s beating her nd cheating on her,... Wah will u say abut dat</t>
-  </si>
-  <si>
-    <t>Why leave a cheating spouse when you can stay and ruin his life</t>
-  </si>
-  <si>
     <t>Never use cheating as an excuse when dating as a woman. If you don't like that attitude, break up with that guy right away since you'll regret it for the rest of your life when you're married.</t>
   </si>
   <si>
-    <t>Lmao better to be a sleeping around woman than be with a "Husband" who goes around disrespecting WIFEE sleeping with anything sleepable. Make everywhere scatter!</t>
-  </si>
-  <si>
-    <t>Hard truth, watch how they will twist this into; he's encouraging cheating.</t>
-  </si>
-  <si>
     <t>A lot of facts here are better imagined than experienced. When you sit down with older ladies who left their husbands for little issues that could be managed, now they're begging for just a night together with a man who doesn't have their time. There's money no companionship.Sad!</t>
   </si>
   <si>
-    <t>Will men please stop cheating for crying out loud!!! Nawa ooo</t>
-  </si>
-  <si>
     <t>Thank you for this word(if you want to leave your husband leave him to be alone) yes leave him to focus on yourself and your children not to go follow another man...if you want to follow another man why bother leaving your husband there are no Saint guys anywhere</t>
   </si>
   <si>
     <t>sometimes wetin dey cause dis cheating na wen man no dey get enough s*x from the partner.</t>
   </si>
   <si>
-    <t>It's the 'if you get caught,I'm sorry for you for me',Knowing fully well men don't forgive cheating lmao</t>
-  </si>
-  <si>
     <t>This advice is doing men more harm than good. When women manage cheating men because there are no better options out there, they start to develop resentment for their partners which usually doesn't end when. Women have started stabbing and setting their cheating partners ablaze.</t>
   </si>
   <si>
-    <t>Read this thread..what we discussed yesterday...Women don't want to accept the truth</t>
-  </si>
-  <si>
     <t>If you must ask for a divorce please do because you are tired and it takes away your peace of mind. Don't divorce because you want to find someone better. If in your being single again you find a partner who later becomes what you prayed for then congratulations. Don't misread</t>
   </si>
   <si>
-    <t>I pity the women who listen to people like you. All these agents of darkness sent to keep people bondage. God that said married people shouldn't commit adultery is stupid while you are wise abi? Instead of advising men to be faithful you're spewing garb. Shame on you...</t>
-  </si>
-  <si>
-    <t>Whichever man who misunderstands this tweet and sees it as a license to cheat ehnn..lolssss. I pity you dear. We will stay o, we won't leave, your punishment will be in later years. Women that can be enduring and yet dangerous. Continue dear, enjoy well now!</t>
-  </si>
-  <si>
     <t>I want ask, why should it always be the women at the receiving end. Do we women look like God that can't make mistakes and always be forgiving one ode that can't control his third leg</t>
   </si>
   <si>
     <t>If a man has the right to cheat just because he wants to, then a woman should also be able to walk away.</t>
   </si>
   <si>
-    <t>I like to mind my business oo.. Cos I have learnt that no matter how men cheat, there is someone dey cherish and won't want to rub their shit on the person. No matter how many babes Dem get, there is that special no1 babe that means alot to them..</t>
-  </si>
-  <si>
     <t>I have always told ladies that the only major reason to leave a relationship or marriage is physical abuse... Every other issues can be manage. John Doe nice writeup</t>
   </si>
   <si>
-    <t>I feel your pain , but even if does as u hv suggested. Man will still remain man in nature.</t>
-  </si>
-  <si>
-    <t>You need to see the way women are bashing your post on Instagram,one girl even said any man that follows you on Twitter is a red flag Truth is always bitter</t>
-  </si>
-  <si>
-    <t>Women. When your man cheat , just tell him that when next he does it again . You will cheat back and see what will happen .</t>
-  </si>
-  <si>
     <t>He is not encouraging men to cheat read again the tweet is about women's reactions went they catch their man cheating not men should cheat</t>
   </si>
   <si>
@@ -598,25 +355,13 @@
     <t>I had a client who filed for divorce bcos a man she was dating asked her to so that they could be free to marry. I finished the case &amp; got the marriage dissolved. Years later, I met d lady that referred her to me &amp; asked her if the man eventually married my client.She said no.</t>
   </si>
   <si>
-    <t>Is it all about servicing and getting serviced just to survive? If she get money nko? Una go just dey think one way. If she wan dey with another man wey get woman nko? What if that's what she want?</t>
-  </si>
-  <si>
     <t>But. The white ladies leave their cheating husband and claim his properties, they have a social system that forces the man to still provide for the kids. We no get am here, yet we wan copy them, say na wokeness.</t>
   </si>
   <si>
     <t>Ladies should not be afraid of change. You don't know how to be alone so you'd rather stay and get infected. If you can't stand it leave Africa there are countries in need of women even though I might not leave my husband due to him cheating.</t>
   </si>
   <si>
-    <t>A sexually active woman will always crave for sex. Question is, if you leave your man, are you gonna look for another or you will stay celibate?</t>
-  </si>
-  <si>
-    <t>You can say it in public that your father is a cheater and sleeps around, you can't say that for your mother. That's all. Thanks for reading</t>
-  </si>
-  <si>
     <t>We all feel hurt when mistreated. So to the men singing praises to this, I hope you maintain the same energy if she cheats back, you totally asked for it, Idk about anyone else but I'd rather leave a cheating man than cheat back on him, I'd be doing a great dishonor to myself,</t>
-  </si>
-  <si>
-    <t>Comrade, please break this thing down for me. You mean side chick turn wife and wife turn side chick Abi na eye dey pain me?</t>
   </si>
 </sst>
 </file>
@@ -974,7 +719,7 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:A201"/>
+  <dimension ref="A1:A116"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
     <row r="1" spans="1:1">
@@ -1557,431 +1302,6 @@
         <v>115</v>
       </c>
     </row>
-    <row r="117" spans="1:1">
-      <c r="A117" t="s">
-        <v>116</v>
-      </c>
-    </row>
-    <row r="118" spans="1:1">
-      <c r="A118" t="s">
-        <v>117</v>
-      </c>
-    </row>
-    <row r="119" spans="1:1">
-      <c r="A119" t="s">
-        <v>118</v>
-      </c>
-    </row>
-    <row r="120" spans="1:1">
-      <c r="A120" t="s">
-        <v>119</v>
-      </c>
-    </row>
-    <row r="121" spans="1:1">
-      <c r="A121" t="s">
-        <v>120</v>
-      </c>
-    </row>
-    <row r="122" spans="1:1">
-      <c r="A122" t="s">
-        <v>121</v>
-      </c>
-    </row>
-    <row r="123" spans="1:1">
-      <c r="A123" t="s">
-        <v>122</v>
-      </c>
-    </row>
-    <row r="124" spans="1:1">
-      <c r="A124" t="s">
-        <v>123</v>
-      </c>
-    </row>
-    <row r="125" spans="1:1">
-      <c r="A125" t="s">
-        <v>124</v>
-      </c>
-    </row>
-    <row r="126" spans="1:1">
-      <c r="A126" t="s">
-        <v>125</v>
-      </c>
-    </row>
-    <row r="127" spans="1:1">
-      <c r="A127" t="s">
-        <v>126</v>
-      </c>
-    </row>
-    <row r="128" spans="1:1">
-      <c r="A128" t="s">
-        <v>127</v>
-      </c>
-    </row>
-    <row r="129" spans="1:1">
-      <c r="A129" t="s">
-        <v>128</v>
-      </c>
-    </row>
-    <row r="130" spans="1:1">
-      <c r="A130" t="s">
-        <v>129</v>
-      </c>
-    </row>
-    <row r="131" spans="1:1">
-      <c r="A131" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="132" spans="1:1">
-      <c r="A132" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="133" spans="1:1">
-      <c r="A133" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="134" spans="1:1">
-      <c r="A134" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="135" spans="1:1">
-      <c r="A135" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="136" spans="1:1">
-      <c r="A136" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="137" spans="1:1">
-      <c r="A137" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="138" spans="1:1">
-      <c r="A138" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="139" spans="1:1">
-      <c r="A139" t="s">
-        <v>138</v>
-      </c>
-    </row>
-    <row r="140" spans="1:1">
-      <c r="A140" t="s">
-        <v>139</v>
-      </c>
-    </row>
-    <row r="141" spans="1:1">
-      <c r="A141" t="s">
-        <v>140</v>
-      </c>
-    </row>
-    <row r="142" spans="1:1">
-      <c r="A142" t="s">
-        <v>141</v>
-      </c>
-    </row>
-    <row r="143" spans="1:1">
-      <c r="A143" t="s">
-        <v>142</v>
-      </c>
-    </row>
-    <row r="144" spans="1:1">
-      <c r="A144" t="s">
-        <v>143</v>
-      </c>
-    </row>
-    <row r="145" spans="1:1">
-      <c r="A145" t="s">
-        <v>144</v>
-      </c>
-    </row>
-    <row r="146" spans="1:1">
-      <c r="A146" t="s">
-        <v>145</v>
-      </c>
-    </row>
-    <row r="147" spans="1:1">
-      <c r="A147" t="s">
-        <v>146</v>
-      </c>
-    </row>
-    <row r="148" spans="1:1">
-      <c r="A148" t="s">
-        <v>147</v>
-      </c>
-    </row>
-    <row r="149" spans="1:1">
-      <c r="A149" t="s">
-        <v>148</v>
-      </c>
-    </row>
-    <row r="150" spans="1:1">
-      <c r="A150" t="s">
-        <v>149</v>
-      </c>
-    </row>
-    <row r="151" spans="1:1">
-      <c r="A151" t="s">
-        <v>150</v>
-      </c>
-    </row>
-    <row r="152" spans="1:1">
-      <c r="A152" t="s">
-        <v>151</v>
-      </c>
-    </row>
-    <row r="153" spans="1:1">
-      <c r="A153" t="s">
-        <v>152</v>
-      </c>
-    </row>
-    <row r="154" spans="1:1">
-      <c r="A154" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="155" spans="1:1">
-      <c r="A155" t="s">
-        <v>154</v>
-      </c>
-    </row>
-    <row r="156" spans="1:1">
-      <c r="A156" t="s">
-        <v>155</v>
-      </c>
-    </row>
-    <row r="157" spans="1:1">
-      <c r="A157" t="s">
-        <v>156</v>
-      </c>
-    </row>
-    <row r="158" spans="1:1">
-      <c r="A158" t="s">
-        <v>157</v>
-      </c>
-    </row>
-    <row r="159" spans="1:1">
-      <c r="A159" t="s">
-        <v>158</v>
-      </c>
-    </row>
-    <row r="160" spans="1:1">
-      <c r="A160" t="s">
-        <v>159</v>
-      </c>
-    </row>
-    <row r="161" spans="1:1">
-      <c r="A161" t="s">
-        <v>160</v>
-      </c>
-    </row>
-    <row r="162" spans="1:1">
-      <c r="A162" t="s">
-        <v>161</v>
-      </c>
-    </row>
-    <row r="163" spans="1:1">
-      <c r="A163" t="s">
-        <v>162</v>
-      </c>
-    </row>
-    <row r="164" spans="1:1">
-      <c r="A164" t="s">
-        <v>163</v>
-      </c>
-    </row>
-    <row r="165" spans="1:1">
-      <c r="A165" t="s">
-        <v>164</v>
-      </c>
-    </row>
-    <row r="166" spans="1:1">
-      <c r="A166" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="167" spans="1:1">
-      <c r="A167" t="s">
-        <v>166</v>
-      </c>
-    </row>
-    <row r="168" spans="1:1">
-      <c r="A168" t="s">
-        <v>167</v>
-      </c>
-    </row>
-    <row r="169" spans="1:1">
-      <c r="A169" t="s">
-        <v>168</v>
-      </c>
-    </row>
-    <row r="170" spans="1:1">
-      <c r="A170" t="s">
-        <v>169</v>
-      </c>
-    </row>
-    <row r="171" spans="1:1">
-      <c r="A171" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="172" spans="1:1">
-      <c r="A172" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="173" spans="1:1">
-      <c r="A173" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="174" spans="1:1">
-      <c r="A174" t="s">
-        <v>173</v>
-      </c>
-    </row>
-    <row r="175" spans="1:1">
-      <c r="A175" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="176" spans="1:1">
-      <c r="A176" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="177" spans="1:1">
-      <c r="A177" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="178" spans="1:1">
-      <c r="A178" t="s">
-        <v>177</v>
-      </c>
-    </row>
-    <row r="179" spans="1:1">
-      <c r="A179" t="s">
-        <v>178</v>
-      </c>
-    </row>
-    <row r="180" spans="1:1">
-      <c r="A180" t="s">
-        <v>179</v>
-      </c>
-    </row>
-    <row r="181" spans="1:1">
-      <c r="A181" t="s">
-        <v>180</v>
-      </c>
-    </row>
-    <row r="182" spans="1:1">
-      <c r="A182" t="s">
-        <v>181</v>
-      </c>
-    </row>
-    <row r="183" spans="1:1">
-      <c r="A183" t="s">
-        <v>182</v>
-      </c>
-    </row>
-    <row r="184" spans="1:1">
-      <c r="A184" t="s">
-        <v>183</v>
-      </c>
-    </row>
-    <row r="185" spans="1:1">
-      <c r="A185" t="s">
-        <v>184</v>
-      </c>
-    </row>
-    <row r="186" spans="1:1">
-      <c r="A186" t="s">
-        <v>185</v>
-      </c>
-    </row>
-    <row r="187" spans="1:1">
-      <c r="A187" t="s">
-        <v>186</v>
-      </c>
-    </row>
-    <row r="188" spans="1:1">
-      <c r="A188" t="s">
-        <v>187</v>
-      </c>
-    </row>
-    <row r="189" spans="1:1">
-      <c r="A189" t="s">
-        <v>188</v>
-      </c>
-    </row>
-    <row r="190" spans="1:1">
-      <c r="A190" t="s">
-        <v>189</v>
-      </c>
-    </row>
-    <row r="191" spans="1:1">
-      <c r="A191" t="s">
-        <v>190</v>
-      </c>
-    </row>
-    <row r="192" spans="1:1">
-      <c r="A192" t="s">
-        <v>191</v>
-      </c>
-    </row>
-    <row r="193" spans="1:1">
-      <c r="A193" t="s">
-        <v>192</v>
-      </c>
-    </row>
-    <row r="194" spans="1:1">
-      <c r="A194" t="s">
-        <v>193</v>
-      </c>
-    </row>
-    <row r="195" spans="1:1">
-      <c r="A195" t="s">
-        <v>194</v>
-      </c>
-    </row>
-    <row r="196" spans="1:1">
-      <c r="A196" t="s">
-        <v>195</v>
-      </c>
-    </row>
-    <row r="197" spans="1:1">
-      <c r="A197" t="s">
-        <v>196</v>
-      </c>
-    </row>
-    <row r="198" spans="1:1">
-      <c r="A198" t="s">
-        <v>197</v>
-      </c>
-    </row>
-    <row r="199" spans="1:1">
-      <c r="A199" t="s">
-        <v>198</v>
-      </c>
-    </row>
-    <row r="200" spans="1:1">
-      <c r="A200" t="s">
-        <v>199</v>
-      </c>
-    </row>
-    <row r="201" spans="1:1">
-      <c r="A201" t="s">
-        <v>200</v>
-      </c>
-    </row>
   </sheetData>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>

</xml_diff>

<commit_message>
strip leading OG pull-quotes from 2 agba rows (paranoid fingerprint audit)
</commit_message>
<xml_diff>
--- a/Topic Relevant Comments/Nigeria/Agba John Doe_Never Leave Marriage Because Husband Cheated.xlsx
+++ b/Topic Relevant Comments/Nigeria/Agba John Doe_Never Leave Marriage Because Husband Cheated.xlsx
@@ -22,7 +22,7 @@
     <t>This is why, when I go on dates. I ask a lot of questions. What's your take on infidelity? Is it possible to stay faithful in a marriage? I'm not saying one cannot fall, but I won't go for someone who already has it in mind to cheat or believes it's normal, even before marrying.</t>
   </si>
   <si>
-    <t>"Except you're done with marriage for good &amp; don't wish to be married again." I belong to this school of thought. For me, infidelity is one of the unpardonable sins.</t>
+    <t>I belong to this school of thought. For me, infidelity is one of the unpardonable sins.</t>
   </si>
   <si>
     <t>Your thread makes it look like men are doing women a favour by getting married to them. Cheating is abnormal, it shows lack of discipline and should never be promoted. If you can't be faithful to her don't marry her. STDs will humble you.</t>
@@ -70,7 +70,7 @@
     <t>The grass is not always greener on the other side. The devil you know is better than the angel you don't. Men cheat because they want to, not because he doesn't respect what you share. Two wrongs don't make a right. If you cheat &amp; get caught, the consequences are different</t>
   </si>
   <si>
-    <t>"A man does not cheat on you because he doesn't find you valuable anymore" Dear Sister, if U believe in marriage please fight for it, consequences of cheating are not the same for a man and woman As the woman you know the odds are against you, don't let SM deceive you</t>
+    <t>Dear Sister, if U believe in marriage please fight for it, consequences of cheating are not the same for a man and woman As the woman you know the odds are against you, don't let SM deceive you</t>
   </si>
   <si>
     <t>This is one falsehood propergated by men to lock women who are unhappy in their marriages due to a cheating spouse. Forgiveness should be done for one's healing but staying is a choice you cannot stay with a serial cheater because he is purportedly the best.</t>

</xml_diff>